<commit_message>
alt text and welcoming fixes
</commit_message>
<xml_diff>
--- a/research/files/openbikeroutesdb.xlsx
+++ b/research/files/openbikeroutesdb.xlsx
@@ -376,7 +376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" style="2" min="1" max="1"/>
@@ -431,7 +431,34 @@
       <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Licence: Creative Commons Zero 1.0 Universal (CC0). We have waived our copyright in this file worldwide. Use it, change it, redistribute it, build on it, sell it. No permission needed and no conditions attached. https://creativecommons.org/publicdomain/zero/1.0/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Attribution is not legally required under CC0, but often requested as a community norm. A citation facilitates transparency and discovery, so thanks in advance!</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Suggested citation: BC Cycle Tourism Society (2026). OpenBikeRoutesDB — route inventory [data set]. Version 2026-06-09. https://bccycletourism.ca/research/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>The research here uses AI assistance (Claude models, Anthropic) for data collection, analysis, and writing. Feel free to ask for more details if you are interested.</t>
         </is>

</xml_diff>

<commit_message>
update after research vet
</commit_message>
<xml_diff>
--- a/research/files/openbikeroutesdb.xlsx
+++ b/research/files/openbikeroutesdb.xlsx
@@ -376,7 +376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" style="2" min="1" max="1"/>
@@ -400,57 +400,57 @@
       <c r="A3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Preliminary — working data, subject to revision.</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>The routes were compiled by hand from route networks' own pages, guidebooks, and tourism organization inventories, and the bibliography is the research we could find about those routes: economic impact studies, visitor surveys, planning documents. Neither file is complete and neither claims to be.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Lengths, surfaces, and terrain are as each route's publisher states them, not measured or verified by us, and a blank cell means we do not know, not that there is nothing to know.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Preliminary — working data, subject to revision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Published 2026-06-09 by BC Cycle Tourism Society.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Questions, corrections, or collaborations: heather@bccycletourism.ca</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>https://bccycletourism.ca/research/</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Licence: Creative Commons Zero 1.0 Universal (CC0). We have waived our copyright in this file worldwide. Use it, change it, redistribute it, build on it, sell it. No permission needed and no conditions attached. https://creativecommons.org/publicdomain/zero/1.0/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Attribution is not legally required under CC0, but often requested as a community norm. A citation facilitates transparency and discovery, so thanks in advance!</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Suggested citation: BC Cycle Tourism Society (2026). OpenBikeRoutesDB — route inventory [data set]. Version 2026-06-09. https://bccycletourism.ca/research/</t>
         </is>
       </c>
     </row>
@@ -458,7 +458,24 @@
       <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Attribution is not legally required under CC0, but often requested as a community norm. A citation facilitates transparency and discovery, so thanks in advance!</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Suggested citation: BC Cycle Tourism Society (2026). OpenBikeRoutesDB — route inventory [data set]. Version 2026-06-09. https://bccycletourism.ca/research/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>The research here uses AI assistance (Claude models, Anthropic) for data collection, analysis, and writing. Feel free to ask for more details if you are interested.</t>
         </is>

</xml_diff>